<commit_message>
added Threat Modeling - Model Analysis training source material
</commit_message>
<xml_diff>
--- a/source/reference_documents/working_material/example system/example system attack surface analysis model.xlsx
+++ b/source/reference_documents/working_material/example system/example system attack surface analysis model.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10413"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10420"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/charles.wilson/Documents/projects/AVCDL/source/reference_documents/working_material/example system/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7598F9F9-FE6D-034F-AE5F-1E1624FF16B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9D8A8D1-1E24-0D4D-8FEF-DED8335159DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10960" yWindow="11700" windowWidth="40860" windowHeight="25120" activeTab="6" xr2:uid="{DEA20EDE-F7A8-FC4F-9F8A-95A2B1030BD3}"/>
+    <workbookView xWindow="24700" yWindow="14780" windowWidth="40860" windowHeight="25120" activeTab="6" xr2:uid="{DEA20EDE-F7A8-FC4F-9F8A-95A2B1030BD3}"/>
   </bookViews>
   <sheets>
     <sheet name="cover sheet" sheetId="7" r:id="rId1"/>
@@ -22,7 +22,7 @@
     <sheet name="4. processes" sheetId="5" r:id="rId7"/>
     <sheet name="legend" sheetId="2" r:id="rId8"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="153">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="154">
   <si>
     <t>DO NOT EDIT THIS PAGE</t>
   </si>
@@ -522,6 +522,9 @@
   <si>
     <t>external</t>
   </si>
+  <si>
+    <t>«</t>
+  </si>
 </sst>
 </file>
 
@@ -530,7 +533,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-409]d\-mmm\-yyyy;@"/>
   </numFmts>
-  <fonts count="17" x14ac:knownFonts="1">
+  <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -639,6 +642,12 @@
       <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Wingdings"/>
+      <charset val="2"/>
     </font>
   </fonts>
   <fills count="4">
@@ -757,6 +766,10 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment textRotation="45"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -776,11 +789,7 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1123,121 +1132,121 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:11" ht="63" x14ac:dyDescent="0.75">
-      <c r="B2" s="24" t="s">
+      <c r="B2" s="28" t="s">
         <v>76</v>
       </c>
-      <c r="C2" s="24"/>
-      <c r="D2" s="24"/>
-      <c r="E2" s="24"/>
-      <c r="F2" s="24"/>
-      <c r="G2" s="24"/>
-      <c r="H2" s="24"/>
-      <c r="I2" s="24"/>
-      <c r="J2" s="24"/>
-      <c r="K2" s="24"/>
+      <c r="C2" s="28"/>
+      <c r="D2" s="28"/>
+      <c r="E2" s="28"/>
+      <c r="F2" s="28"/>
+      <c r="G2" s="28"/>
+      <c r="H2" s="28"/>
+      <c r="I2" s="28"/>
+      <c r="J2" s="28"/>
+      <c r="K2" s="28"/>
     </row>
     <row r="4" spans="2:11" ht="32" x14ac:dyDescent="0.4">
       <c r="B4" s="8" t="s">
         <v>50</v>
       </c>
       <c r="C4" s="6"/>
-      <c r="D4" s="26" t="s">
+      <c r="D4" s="30" t="s">
         <v>50</v>
       </c>
-      <c r="E4" s="26"/>
-      <c r="F4" s="26"/>
-      <c r="G4" s="26"/>
-      <c r="H4" s="26"/>
-      <c r="I4" s="26"/>
-      <c r="J4" s="26"/>
+      <c r="E4" s="30"/>
+      <c r="F4" s="30"/>
+      <c r="G4" s="30"/>
+      <c r="H4" s="30"/>
+      <c r="I4" s="30"/>
+      <c r="J4" s="30"/>
     </row>
     <row r="6" spans="2:11" ht="32" x14ac:dyDescent="0.4">
       <c r="B6" s="8" t="s">
         <v>61</v>
       </c>
       <c r="C6" s="6"/>
-      <c r="D6" s="26" t="s">
+      <c r="D6" s="30" t="s">
         <v>61</v>
       </c>
-      <c r="E6" s="26"/>
-      <c r="F6" s="26"/>
-      <c r="G6" s="26"/>
-      <c r="H6" s="26"/>
-      <c r="I6" s="26"/>
-      <c r="J6" s="26"/>
+      <c r="E6" s="30"/>
+      <c r="F6" s="30"/>
+      <c r="G6" s="30"/>
+      <c r="H6" s="30"/>
+      <c r="I6" s="30"/>
+      <c r="J6" s="30"/>
     </row>
     <row r="8" spans="2:11" ht="32" x14ac:dyDescent="0.4">
       <c r="B8" s="8" t="s">
         <v>80</v>
       </c>
       <c r="C8" s="6"/>
-      <c r="D8" s="26"/>
-      <c r="E8" s="26"/>
-      <c r="F8" s="26"/>
-      <c r="G8" s="26"/>
-      <c r="H8" s="26"/>
-      <c r="I8" s="26"/>
-      <c r="J8" s="26"/>
+      <c r="D8" s="30"/>
+      <c r="E8" s="30"/>
+      <c r="F8" s="30"/>
+      <c r="G8" s="30"/>
+      <c r="H8" s="30"/>
+      <c r="I8" s="30"/>
+      <c r="J8" s="30"/>
     </row>
     <row r="10" spans="2:11" ht="32" x14ac:dyDescent="0.4">
       <c r="B10" s="8" t="s">
         <v>51</v>
       </c>
       <c r="C10" s="6"/>
-      <c r="D10" s="27" t="s">
+      <c r="D10" s="31" t="s">
         <v>51</v>
       </c>
-      <c r="E10" s="27"/>
-      <c r="F10" s="27"/>
-      <c r="G10" s="27"/>
-      <c r="H10" s="27"/>
-      <c r="I10" s="27"/>
-      <c r="J10" s="27"/>
+      <c r="E10" s="31"/>
+      <c r="F10" s="31"/>
+      <c r="G10" s="31"/>
+      <c r="H10" s="31"/>
+      <c r="I10" s="31"/>
+      <c r="J10" s="31"/>
     </row>
     <row r="12" spans="2:11" ht="32" x14ac:dyDescent="0.4">
       <c r="B12" s="8" t="s">
         <v>52</v>
       </c>
       <c r="C12" s="6"/>
-      <c r="D12" s="27" t="s">
+      <c r="D12" s="31" t="s">
         <v>52</v>
       </c>
-      <c r="E12" s="27"/>
-      <c r="F12" s="27"/>
-      <c r="G12" s="27"/>
-      <c r="H12" s="27"/>
-      <c r="I12" s="27"/>
-      <c r="J12" s="27"/>
+      <c r="E12" s="31"/>
+      <c r="F12" s="31"/>
+      <c r="G12" s="31"/>
+      <c r="H12" s="31"/>
+      <c r="I12" s="31"/>
+      <c r="J12" s="31"/>
     </row>
     <row r="14" spans="2:11" ht="32" x14ac:dyDescent="0.4">
       <c r="B14" s="8" t="s">
         <v>77</v>
       </c>
       <c r="C14" s="6"/>
-      <c r="D14" s="27" t="s">
+      <c r="D14" s="31" t="s">
         <v>77</v>
       </c>
-      <c r="E14" s="27"/>
-      <c r="F14" s="27"/>
-      <c r="G14" s="27"/>
-      <c r="H14" s="27"/>
-      <c r="I14" s="27"/>
-      <c r="J14" s="27"/>
+      <c r="E14" s="31"/>
+      <c r="F14" s="31"/>
+      <c r="G14" s="31"/>
+      <c r="H14" s="31"/>
+      <c r="I14" s="31"/>
+      <c r="J14" s="31"/>
     </row>
     <row r="16" spans="2:11" ht="32" x14ac:dyDescent="0.4">
       <c r="B16" s="8" t="s">
         <v>53</v>
       </c>
       <c r="C16" s="6"/>
-      <c r="D16" s="28">
+      <c r="D16" s="32">
         <v>36765</v>
       </c>
-      <c r="E16" s="28"/>
-      <c r="F16" s="28"/>
-      <c r="G16" s="28"/>
-      <c r="H16" s="28"/>
-      <c r="I16" s="28"/>
-      <c r="J16" s="28"/>
+      <c r="E16" s="32"/>
+      <c r="F16" s="32"/>
+      <c r="G16" s="32"/>
+      <c r="H16" s="32"/>
+      <c r="I16" s="32"/>
+      <c r="J16" s="32"/>
     </row>
     <row r="18" spans="2:11" ht="32" x14ac:dyDescent="0.4">
       <c r="B18" s="8" t="s">
@@ -1254,18 +1263,18 @@
       <c r="D19" s="6"/>
     </row>
     <row r="20" spans="2:11" ht="32" x14ac:dyDescent="0.4">
-      <c r="B20" s="25" t="s">
+      <c r="B20" s="29" t="s">
         <v>78</v>
       </c>
-      <c r="C20" s="25"/>
-      <c r="D20" s="25"/>
-      <c r="E20" s="25"/>
-      <c r="F20" s="25"/>
-      <c r="G20" s="25"/>
-      <c r="H20" s="25"/>
-      <c r="I20" s="25"/>
-      <c r="J20" s="25"/>
-      <c r="K20" s="25"/>
+      <c r="C20" s="29"/>
+      <c r="D20" s="29"/>
+      <c r="E20" s="29"/>
+      <c r="F20" s="29"/>
+      <c r="G20" s="29"/>
+      <c r="H20" s="29"/>
+      <c r="I20" s="29"/>
+      <c r="J20" s="29"/>
+      <c r="K20" s="29"/>
     </row>
   </sheetData>
   <mergeCells count="9">
@@ -1310,11 +1319,11 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:7" ht="63" x14ac:dyDescent="0.75">
-      <c r="B2" s="29" t="s">
+      <c r="B2" s="33" t="s">
         <v>62</v>
       </c>
-      <c r="C2" s="29"/>
-      <c r="D2" s="29"/>
+      <c r="C2" s="33"/>
+      <c r="D2" s="33"/>
       <c r="E2" s="7"/>
       <c r="F2" s="7"/>
       <c r="G2" s="7"/>
@@ -1433,11 +1442,11 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:7" ht="63" x14ac:dyDescent="0.75">
-      <c r="B2" s="29" t="s">
+      <c r="B2" s="33" t="s">
         <v>66</v>
       </c>
-      <c r="C2" s="29"/>
-      <c r="D2" s="29"/>
+      <c r="C2" s="33"/>
+      <c r="D2" s="33"/>
       <c r="E2" s="7"/>
       <c r="F2" s="7"/>
       <c r="G2" s="7"/>
@@ -1548,30 +1557,30 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="2" spans="2:10" ht="63" x14ac:dyDescent="0.75">
-      <c r="B2" s="29" t="s">
+      <c r="B2" s="33" t="s">
         <v>55</v>
       </c>
-      <c r="C2" s="29"/>
-      <c r="D2" s="29"/>
-      <c r="E2" s="29"/>
-      <c r="F2" s="29"/>
-      <c r="G2" s="29"/>
-      <c r="H2" s="29"/>
-      <c r="I2" s="29"/>
-      <c r="J2" s="29"/>
+      <c r="C2" s="33"/>
+      <c r="D2" s="33"/>
+      <c r="E2" s="33"/>
+      <c r="F2" s="33"/>
+      <c r="G2" s="33"/>
+      <c r="H2" s="33"/>
+      <c r="I2" s="33"/>
+      <c r="J2" s="33"/>
     </row>
     <row r="5" spans="2:10" ht="27" x14ac:dyDescent="0.35">
-      <c r="B5" s="30" t="s">
+      <c r="B5" s="34" t="s">
         <v>57</v>
       </c>
-      <c r="C5" s="30"/>
-      <c r="D5" s="30"/>
-      <c r="E5" s="30"/>
-      <c r="F5" s="30"/>
-      <c r="G5" s="30"/>
-      <c r="H5" s="30"/>
-      <c r="I5" s="30"/>
-      <c r="J5" s="30"/>
+      <c r="C5" s="34"/>
+      <c r="D5" s="34"/>
+      <c r="E5" s="34"/>
+      <c r="F5" s="34"/>
+      <c r="G5" s="34"/>
+      <c r="H5" s="34"/>
+      <c r="I5" s="34"/>
+      <c r="J5" s="34"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1598,15 +1607,15 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:12" ht="63" x14ac:dyDescent="0.75">
-      <c r="B2" s="29" t="s">
+      <c r="B2" s="33" t="s">
         <v>58</v>
       </c>
-      <c r="C2" s="29"/>
-      <c r="D2" s="29"/>
-      <c r="E2" s="29"/>
-      <c r="F2" s="29"/>
-      <c r="G2" s="29"/>
-      <c r="H2" s="29"/>
+      <c r="C2" s="33"/>
+      <c r="D2" s="33"/>
+      <c r="E2" s="33"/>
+      <c r="F2" s="33"/>
+      <c r="G2" s="33"/>
+      <c r="H2" s="33"/>
       <c r="I2" s="7"/>
       <c r="J2" s="7"/>
       <c r="K2" s="7"/>
@@ -1686,7 +1695,7 @@
       <c r="B7" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="C7" s="31" t="s">
+      <c r="C7" t="s">
         <v>109</v>
       </c>
       <c r="D7" s="3" t="s">
@@ -1749,7 +1758,7 @@
       <c r="B10" s="3" t="s">
         <v>91</v>
       </c>
-      <c r="C10" s="32" t="s">
+      <c r="C10" s="24" t="s">
         <v>103</v>
       </c>
       <c r="D10" s="3" t="s">
@@ -1977,15 +1986,15 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:12" ht="63" x14ac:dyDescent="0.75">
-      <c r="B2" s="29" t="s">
+      <c r="B2" s="33" t="s">
         <v>60</v>
       </c>
-      <c r="C2" s="29"/>
-      <c r="D2" s="29"/>
-      <c r="E2" s="29"/>
-      <c r="F2" s="29"/>
-      <c r="G2" s="29"/>
-      <c r="H2" s="29"/>
+      <c r="C2" s="33"/>
+      <c r="D2" s="33"/>
+      <c r="E2" s="33"/>
+      <c r="F2" s="33"/>
+      <c r="G2" s="33"/>
+      <c r="H2" s="33"/>
       <c r="I2" s="7"/>
       <c r="K2" s="7"/>
       <c r="L2" s="7"/>
@@ -2203,7 +2212,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{78F199F4-5379-E940-BD25-0601604382B3}">
-  <dimension ref="A2:L20"/>
+  <dimension ref="A2:L30"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="16.83203125" bestFit="1" customWidth="1"/>
@@ -2216,16 +2225,16 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:12" ht="63" x14ac:dyDescent="0.75">
-      <c r="B2" s="29" t="s">
+      <c r="B2" s="33" t="s">
         <v>59</v>
       </c>
-      <c r="C2" s="29"/>
-      <c r="D2" s="29"/>
-      <c r="E2" s="29"/>
-      <c r="F2" s="29"/>
-      <c r="G2" s="29"/>
-      <c r="H2" s="29"/>
-      <c r="I2" s="29"/>
+      <c r="C2" s="33"/>
+      <c r="D2" s="33"/>
+      <c r="E2" s="33"/>
+      <c r="F2" s="33"/>
+      <c r="G2" s="33"/>
+      <c r="H2" s="33"/>
+      <c r="I2" s="33"/>
       <c r="J2" s="7"/>
       <c r="K2" s="7"/>
       <c r="L2" s="7"/>
@@ -2258,10 +2267,10 @@
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="B5" s="33" t="s">
+      <c r="B5" s="25" t="s">
         <v>135</v>
       </c>
-      <c r="C5" s="33" t="s">
+      <c r="C5" s="25" t="s">
         <v>136</v>
       </c>
       <c r="D5" s="3" t="s">
@@ -2270,7 +2279,7 @@
       <c r="E5" s="5" t="s">
         <v>144</v>
       </c>
-      <c r="F5" s="34" t="s">
+      <c r="F5" s="26" t="s">
         <v>141</v>
       </c>
       <c r="G5" s="5" t="s">
@@ -2282,10 +2291,10 @@
       <c r="I5" s="5"/>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="B6" s="33" t="s">
+      <c r="B6" s="25" t="s">
         <v>137</v>
       </c>
-      <c r="C6" s="33" t="s">
+      <c r="C6" s="25" t="s">
         <v>138</v>
       </c>
       <c r="D6" s="3" t="s">
@@ -2294,7 +2303,7 @@
       <c r="E6" s="5" t="s">
         <v>144</v>
       </c>
-      <c r="F6" s="34" t="s">
+      <c r="F6" s="26" t="s">
         <v>142</v>
       </c>
       <c r="G6" s="5" t="s">
@@ -2306,10 +2315,10 @@
       <c r="I6" s="5"/>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="B7" s="33" t="s">
+      <c r="B7" s="25" t="s">
         <v>139</v>
       </c>
-      <c r="C7" s="33" t="s">
+      <c r="C7" s="25" t="s">
         <v>140</v>
       </c>
       <c r="D7" s="3" t="s">
@@ -2318,7 +2327,7 @@
       <c r="E7" s="5" t="s">
         <v>145</v>
       </c>
-      <c r="F7" s="34" t="s">
+      <c r="F7" s="26" t="s">
         <v>143</v>
       </c>
       <c r="G7" s="5" t="s">
@@ -2458,6 +2467,14 @@
       <c r="G20" s="5"/>
       <c r="H20" s="5"/>
       <c r="I20" s="5"/>
+    </row>
+    <row r="29" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="F29" s="35"/>
+    </row>
+    <row r="30" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="G30" t="s">
+        <v>153</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2512,7 +2529,7 @@
       <c r="E1" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="F1" s="35" t="s">
+      <c r="F1" s="27" t="s">
         <v>150</v>
       </c>
     </row>

</xml_diff>